<commit_message>
更新 2026-08-10 風險新聞明細（2026-08-10 10:36）
</commit_message>
<xml_diff>
--- a/risk_news_daily/2026-08-10.xlsx
+++ b/risk_news_daily/2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險新聞" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$O$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$P$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O88"/>
+  <dimension ref="A1:P88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="80" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -524,6 +525,11 @@
           <t>已人工覆核</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -570,7 +576,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -593,6 +599,9 @@
         </is>
       </c>
       <c r="O2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -666,6 +675,9 @@
       <c r="O3" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -737,6 +749,9 @@
       <c r="O4" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -808,6 +823,9 @@
       <c r="O5" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P5" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -879,6 +897,9 @@
       <c r="O6" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -950,6 +971,9 @@
       <c r="O7" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1021,6 +1045,9 @@
       <c r="O8" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P8" s="2" t="n">
+        <v>38700750</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1092,6 +1119,9 @@
       <c r="O9" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1163,6 +1193,9 @@
       <c r="O10" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1234,6 +1267,9 @@
       <c r="O11" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1305,6 +1341,9 @@
       <c r="O12" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1376,6 +1415,9 @@
       <c r="O13" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1447,6 +1489,9 @@
       <c r="O14" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P14" s="2" t="n">
+        <v>34300700</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1518,6 +1563,9 @@
       <c r="O15" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P15" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1589,6 +1637,9 @@
       <c r="O16" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1660,6 +1711,9 @@
       <c r="O17" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P17" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1731,6 +1785,9 @@
       <c r="O18" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P18" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1802,6 +1859,9 @@
       <c r="O19" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P19" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1873,6 +1933,9 @@
       <c r="O20" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P20" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1944,6 +2007,9 @@
       <c r="O21" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P21" s="2" t="n">
+        <v>38700750</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2015,6 +2081,9 @@
       <c r="O22" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P22" s="2" t="n">
+        <v>95500380</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2086,6 +2155,9 @@
       <c r="O23" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P23" s="2" t="n">
+        <v>10900000</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2157,6 +2229,9 @@
       <c r="O24" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2228,6 +2303,9 @@
       <c r="O25" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2299,6 +2377,9 @@
       <c r="O26" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P26" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2370,6 +2451,9 @@
       <c r="O27" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2441,6 +2525,9 @@
       <c r="O28" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P28" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2512,6 +2599,9 @@
       <c r="O29" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P29" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2583,6 +2673,9 @@
       <c r="O30" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2654,6 +2747,9 @@
       <c r="O31" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2725,6 +2821,9 @@
       <c r="O32" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P32" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2796,6 +2895,9 @@
       <c r="O33" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P33" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2867,6 +2969,9 @@
       <c r="O34" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2938,6 +3043,9 @@
       <c r="O35" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P35" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3009,6 +3117,9 @@
       <c r="O36" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P36" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3080,6 +3191,9 @@
       <c r="O37" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P37" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3151,6 +3265,9 @@
       <c r="O38" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P38" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3222,6 +3339,9 @@
       <c r="O39" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P39" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3293,6 +3413,9 @@
       <c r="O40" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P40" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3364,6 +3487,9 @@
       <c r="O41" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P41" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3435,6 +3561,9 @@
       <c r="O42" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P42" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3506,6 +3635,9 @@
       <c r="O43" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P43" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3577,6 +3709,9 @@
       <c r="O44" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P44" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3648,6 +3783,9 @@
       <c r="O45" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P45" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3719,6 +3857,9 @@
       <c r="O46" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P46" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3790,6 +3931,9 @@
       <c r="O47" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P47" s="2" t="n">
+        <v>10900000</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3861,6 +4005,9 @@
       <c r="O48" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P48" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3932,6 +4079,9 @@
       <c r="O49" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P49" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4003,6 +4153,9 @@
       <c r="O50" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P50" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4074,6 +4227,9 @@
       <c r="O51" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P51" s="2" t="n">
+        <v>95500380</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4145,6 +4301,9 @@
       <c r="O52" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P52" s="2" t="n">
+        <v>10900000</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4216,6 +4375,9 @@
       <c r="O53" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P53" s="2" t="n">
+        <v>293100070</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4287,6 +4449,9 @@
       <c r="O54" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P54" s="2" t="n">
+        <v>6200000</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4358,6 +4523,9 @@
       <c r="O55" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4429,6 +4597,9 @@
       <c r="O56" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P56" s="2" t="n">
+        <v>50100008</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4500,6 +4671,9 @@
       <c r="O57" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P57" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4571,6 +4745,9 @@
       <c r="O58" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P58" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4642,6 +4819,9 @@
       <c r="O59" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P59" s="2" t="n">
+        <v>22304000</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4713,6 +4893,9 @@
       <c r="O60" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P60" s="2" t="n">
+        <v>10900000</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4784,6 +4967,9 @@
       <c r="O61" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P61" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4855,6 +5041,9 @@
       <c r="O62" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P62" s="2" t="n">
+        <v>6200000</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4926,6 +5115,9 @@
       <c r="O63" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P63" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4997,6 +5189,9 @@
       <c r="O64" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P64" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5068,6 +5263,9 @@
       <c r="O65" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P65" s="2" t="n">
+        <v>6200000</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5139,6 +5337,9 @@
       <c r="O66" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P66" s="2" t="n">
+        <v>6200000</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5210,6 +5411,9 @@
       <c r="O67" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P67" s="2" t="n">
+        <v>6200000</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5281,6 +5485,9 @@
       <c r="O68" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P68" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5352,6 +5559,9 @@
       <c r="O69" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P69" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5423,6 +5633,9 @@
       <c r="O70" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P70" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5494,6 +5707,9 @@
       <c r="O71" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P71" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5565,6 +5781,9 @@
       <c r="O72" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P72" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5636,6 +5855,9 @@
       <c r="O73" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P73" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5707,6 +5929,9 @@
       <c r="O74" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P74" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5778,6 +6003,9 @@
       <c r="O75" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P75" s="2" t="n">
+        <v>163090500</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5849,6 +6077,9 @@
       <c r="O76" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P76" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5920,6 +6151,9 @@
       <c r="O77" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P77" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5991,6 +6225,9 @@
       <c r="O78" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P78" s="2" t="n">
+        <v>163090500</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6062,6 +6299,9 @@
       <c r="O79" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P79" s="2" t="n">
+        <v>38700750</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6133,6 +6373,9 @@
       <c r="O80" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P80" s="2" t="n">
+        <v>95500380</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6204,6 +6447,9 @@
       <c r="O81" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P81" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6275,6 +6521,9 @@
       <c r="O82" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P82" s="2" t="n">
+        <v>163090500</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6346,6 +6595,9 @@
       <c r="O83" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P83" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6417,6 +6669,9 @@
       <c r="O84" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P84" s="2" t="n">
+        <v>163090500</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6488,6 +6743,9 @@
       <c r="O85" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P85" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6559,6 +6817,9 @@
       <c r="O86" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P86" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6630,6 +6891,9 @@
       <c r="O87" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P87" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6701,9 +6965,12 @@
       <c r="O88" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P88" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O88"/>
+  <autoFilter ref="A1:P88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>